<commit_message>
Refinando título da hero: Duas linhas e gradiente prateado escuro
</commit_message>
<xml_diff>
--- a/assets/catalogo_link360.xlsx
+++ b/assets/catalogo_link360.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📦 Catálogo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📖 Instruções" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📊 Resumo" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="📦 Catálogo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="📖 Instruções" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="📊 Resumo" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,8 +73,24 @@
       <color rgb="001A1A2E"/>
       <sz val="14"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <color rgb="FF888888"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FF2E7D32"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFE65100"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -131,8 +147,33 @@
         <fgColor rgb="00495057"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1A1F3D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF8E7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF3E0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -154,11 +195,69 @@
         <color rgb="00DEE2E6"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00DEE2E6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00DEE2E6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00DEE2E6"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00DEE2E6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00DEE2E6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00DEE2E6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00DEE2E6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00DEE2E6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00DDDDDD"/>
+      </left>
+      <right style="thin">
+        <color rgb="00DDDDDD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00DDDDDD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00DDDDDD"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -226,6 +325,41 @@
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -600,23 +734,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:P34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="38" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -627,1932 +763,1894 @@
       </c>
     </row>
     <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="23" t="inlineStr">
         <is>
           <t>Nome do Produto *</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="23" t="inlineStr">
         <is>
           <t>Categoria *</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="23" t="inlineStr">
         <is>
           <t>Velocidade Máx.</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="23" t="inlineStr">
         <is>
           <t>Potência (Motor)</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="23" t="inlineStr">
         <is>
           <t>Autonomia</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="23" t="inlineStr">
         <is>
           <t>Descrição *</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="23" t="inlineStr">
         <is>
           <t>🖼️ Imagem Destaque (URL)</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="23" t="inlineStr">
         <is>
           <t>Imagem 2 (URL)</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J2" s="23" t="inlineStr">
         <is>
           <t>Imagem 3 (URL)</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="K2" s="23" t="inlineStr">
         <is>
           <t>Link do Produto (URL)</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="L2" s="23" t="inlineStr">
         <is>
           <t>Preço (R$)</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M2" s="23" t="inlineStr">
+        <is>
+          <t>Preço Parcelado</t>
+        </is>
+      </c>
+      <c r="N2" s="23" t="inlineStr">
+        <is>
+          <t>Badge / Tag</t>
+        </is>
+      </c>
+      <c r="O2" s="23" t="inlineStr">
         <is>
           <t>🔥 Oferta em Destaque?</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="P2" s="23" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="4" t="n">
+    <row r="3" ht="52" customHeight="1">
+      <c r="A3" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Giga</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="24" t="inlineStr">
         <is>
           <t>Autopropelidos</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="24" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="24" t="inlineStr">
         <is>
           <t>1000 W</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="24" t="inlineStr">
         <is>
           <t>40 km</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="G3" s="25" t="inlineStr">
         <is>
           <t>Frente agressiva, farol e setas em LED e painel digital futurista. Escolha de quem quer sair do óbvio, chegar em silêncio e causar impacto.</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/Giga_modelo.webp</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr"/>
-      <c r="J3" s="5" t="inlineStr"/>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="I3" s="24" t="inlineStr"/>
+      <c r="J3" s="24" t="inlineStr"/>
+      <c r="K3" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/giga</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr"/>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="L3" s="24" t="inlineStr"/>
+      <c r="M3" s="24" t="inlineStr"/>
+      <c r="N3" s="24" t="inlineStr">
+        <is>
+          <t>Sem CNH</t>
+        </is>
+      </c>
+      <c r="O3" s="26" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="P3" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="7" t="n">
+    <row r="4" ht="52" customHeight="1">
+      <c r="A4" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>JET MAX</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="28" t="inlineStr">
         <is>
           <t>Autopropelidos</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="E4" s="28" t="inlineStr">
         <is>
           <t>1000 W</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="F4" s="28" t="inlineStr">
         <is>
           <t>55 km</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>Visual esportivo de scooter robusta com tecnologia e conforto. Motor 1000W com 55 km de autonomia.</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="G4" s="29" t="inlineStr">
+        <is>
+          <t>Visual esportivo de scooter robusta com tecnologia e conforto. Motor 1000W e maior autonomia da linha: 55 km por carga.</t>
+        </is>
+      </c>
+      <c r="H4" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/JET-MAX-_-Oficial-2_b.webp</t>
         </is>
       </c>
-      <c r="I4" s="8" t="inlineStr"/>
-      <c r="J4" s="8" t="inlineStr"/>
-      <c r="K4" s="8" t="inlineStr">
+      <c r="I4" s="28" t="inlineStr"/>
+      <c r="J4" s="28" t="inlineStr"/>
+      <c r="K4" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/jet-max</t>
         </is>
       </c>
-      <c r="L4" s="7" t="inlineStr"/>
-      <c r="M4" s="7" t="inlineStr">
+      <c r="L4" s="28" t="inlineStr"/>
+      <c r="M4" s="28" t="inlineStr"/>
+      <c r="N4" s="28" t="inlineStr">
+        <is>
+          <t>Sem CNH</t>
+        </is>
+      </c>
+      <c r="O4" s="30" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N4" s="7" t="inlineStr">
+      <c r="P4" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="4" t="n">
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>X12</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="24" t="inlineStr">
         <is>
           <t>Autopropelidos</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="24" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="24" t="inlineStr">
         <is>
           <t>1000 W</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="24" t="inlineStr">
         <is>
           <t>40 km</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Scooter elétrica que redefine mobilidade urbana. Compacta, potente e tecnológica com 1000W e até 50 km de autonomia.</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="G5" s="25" t="inlineStr">
+        <is>
+          <t>Scooter elétrica que redefine mobilidade urbana. Compacta, potente e tecnológica com 1000W e até 40 km de autonomia.</t>
+        </is>
+      </c>
+      <c r="H5" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/10/x12b.webp</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr"/>
-      <c r="J5" s="5" t="inlineStr"/>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="I5" s="24" t="inlineStr"/>
+      <c r="J5" s="24" t="inlineStr"/>
+      <c r="K5" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/x12/</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr"/>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="L5" s="24" t="inlineStr"/>
+      <c r="M5" s="24" t="inlineStr"/>
+      <c r="N5" s="24" t="inlineStr">
+        <is>
+          <t>Sem CNH</t>
+        </is>
+      </c>
+      <c r="O5" s="26" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="P5" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="7" t="n">
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="28" t="inlineStr">
         <is>
           <t>BOB</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="28" t="inlineStr">
         <is>
           <t>Autopropelidos</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="28" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="28" t="inlineStr">
         <is>
           <t>1000 W</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="28" t="inlineStr">
         <is>
           <t>40 km</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>Posição confortável, plataforma baixa, assento amplo com espaço para carona e encosto traseiro.</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="G6" s="29" t="inlineStr">
+        <is>
+          <t>Posição confortável, plataforma baixa, assento amplo com espaço para carona e encosto traseiro. Ideal para o dia a dia urbano.</t>
+        </is>
+      </c>
+      <c r="H6" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/10/bob_1.webp</t>
         </is>
       </c>
-      <c r="I6" s="8" t="inlineStr"/>
-      <c r="J6" s="8" t="inlineStr"/>
-      <c r="K6" s="8" t="inlineStr">
+      <c r="I6" s="28" t="inlineStr"/>
+      <c r="J6" s="28" t="inlineStr"/>
+      <c r="K6" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/bob</t>
         </is>
       </c>
-      <c r="L6" s="7" t="inlineStr"/>
-      <c r="M6" s="7" t="inlineStr">
+      <c r="L6" s="28" t="inlineStr"/>
+      <c r="M6" s="28" t="inlineStr"/>
+      <c r="N6" s="28" t="inlineStr">
+        <is>
+          <t>Sem CNH</t>
+        </is>
+      </c>
+      <c r="O6" s="30" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N6" s="7" t="inlineStr">
+      <c r="P6" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="4" t="n">
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>JET</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="24" t="inlineStr">
         <is>
           <t>Autopropelidos</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="24" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="24" t="inlineStr">
         <is>
           <t>1000 W</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="24" t="inlineStr">
         <is>
           <t>40 km</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Visual agressivo, zero burocracia: ligou, acelerou, chegou.</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="G7" s="25" t="inlineStr">
+        <is>
+          <t>Design esportivo e bateria de lítio removível. Para quem quer estilo, agilidade e zero burocracia no trânsito.</t>
+        </is>
+      </c>
+      <c r="H7" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/10/JET_1-1.webp</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr"/>
-      <c r="J7" s="5" t="inlineStr"/>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="I7" s="24" t="inlineStr"/>
+      <c r="J7" s="24" t="inlineStr"/>
+      <c r="K7" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/jet</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr"/>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="L7" s="24" t="inlineStr"/>
+      <c r="M7" s="24" t="inlineStr"/>
+      <c r="N7" s="24" t="inlineStr">
+        <is>
+          <t>Sem CNH</t>
+        </is>
+      </c>
+      <c r="O7" s="26" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="P7" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="7" t="n">
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="28" t="inlineStr">
         <is>
           <t>Joyzinha</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="28" t="inlineStr">
         <is>
           <t>Autopropelidos</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="28" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="28" t="inlineStr">
         <is>
           <t>600 W</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="28" t="inlineStr">
         <is>
           <t>40 km</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>Design para o dia a dia, parceira ideal para trabalho, faculdade ou passeio na orla.</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="G8" s="29" t="inlineStr">
+        <is>
+          <t>Design compacto para o dia a dia. Parceira ideal para trabalho, faculdade ou passeio na orla — leve e econômica.</t>
+        </is>
+      </c>
+      <c r="H8" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/5.webp</t>
         </is>
       </c>
-      <c r="I8" s="8" t="inlineStr"/>
-      <c r="J8" s="8" t="inlineStr"/>
-      <c r="K8" s="8" t="inlineStr">
+      <c r="I8" s="28" t="inlineStr"/>
+      <c r="J8" s="28" t="inlineStr"/>
+      <c r="K8" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/joyzinha</t>
         </is>
       </c>
-      <c r="L8" s="7" t="inlineStr"/>
-      <c r="M8" s="7" t="inlineStr">
+      <c r="L8" s="28" t="inlineStr"/>
+      <c r="M8" s="28" t="inlineStr"/>
+      <c r="N8" s="28" t="inlineStr">
+        <is>
+          <t>Sem CNH</t>
+        </is>
+      </c>
+      <c r="O8" s="30" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N8" s="7" t="inlineStr">
+      <c r="P8" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="4" t="n">
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>Joy Classic</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="24" t="inlineStr">
         <is>
           <t>Autopropelidos</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="24" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="24" t="inlineStr">
         <is>
           <t>600 W</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" s="24" t="inlineStr">
         <is>
           <t>40 km</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>Estilo clássico, conforto de sobra e autonomia para o seu dia.</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="G9" s="25" t="inlineStr">
+        <is>
+          <t>Estilo clássico, conforto de sobra e autonomia suficiente para o seu dia. Silencioso, econômico e sem emplacamento.</t>
+        </is>
+      </c>
+      <c r="H9" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/10/JOY-CLASSIC-_1-1.webp</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="5" t="inlineStr"/>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="I9" s="24" t="inlineStr"/>
+      <c r="J9" s="24" t="inlineStr"/>
+      <c r="K9" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/joy-classic</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr"/>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="L9" s="24" t="inlineStr"/>
+      <c r="M9" s="24" t="inlineStr"/>
+      <c r="N9" s="24" t="inlineStr">
+        <is>
+          <t>Sem CNH</t>
+        </is>
+      </c>
+      <c r="O9" s="26" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="P9" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="7" t="n">
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="28" t="inlineStr">
         <is>
           <t>Joy Super</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="28" t="inlineStr">
         <is>
           <t>Autopropelidos</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="28" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="28" t="inlineStr">
         <is>
           <t>800 W</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="F10" s="28" t="inlineStr">
         <is>
           <t>40 km</t>
         </is>
       </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>Visual agressivo, zero burocracia: ligou, acelerou, chegou.</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="G10" s="29" t="inlineStr">
+        <is>
+          <t>Motor 800W com tração firme e visual marcante. Mais potência que o clássico, mesma praticidade sem CNH.</t>
+        </is>
+      </c>
+      <c r="H10" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/10/JOY-SUPER-1-1.webp</t>
         </is>
       </c>
-      <c r="I10" s="8" t="inlineStr"/>
-      <c r="J10" s="8" t="inlineStr"/>
-      <c r="K10" s="8" t="inlineStr">
+      <c r="I10" s="28" t="inlineStr"/>
+      <c r="J10" s="28" t="inlineStr"/>
+      <c r="K10" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/joy-super</t>
         </is>
       </c>
-      <c r="L10" s="7" t="inlineStr"/>
-      <c r="M10" s="7" t="inlineStr">
+      <c r="L10" s="28" t="inlineStr"/>
+      <c r="M10" s="28" t="inlineStr"/>
+      <c r="N10" s="28" t="inlineStr">
+        <is>
+          <t>Sem CNH</t>
+        </is>
+      </c>
+      <c r="O10" s="30" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N10" s="7" t="inlineStr">
+      <c r="P10" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="4" t="n">
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="24" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>MC20 Mini</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="24" t="inlineStr">
         <is>
           <t>Autopropelidos</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="24" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="24" t="inlineStr">
         <is>
           <t>1000 W</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" s="24" t="inlineStr">
         <is>
           <t>40 km</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>Farol FULL LED, freio a disco hidráulico, bateria removível turbo 5A, suporta até 180 kg.</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="G11" s="25" t="inlineStr">
+        <is>
+          <t>Farol FULL LED, freio a disco hidráulico, bateria removível turbo 5A. Suporta até 180 kg — robusto de verdade.</t>
+        </is>
+      </c>
+      <c r="H11" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/10/MC20-1-1.webp</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="5" t="inlineStr"/>
-      <c r="K11" s="5" t="inlineStr">
+      <c r="I11" s="24" t="inlineStr"/>
+      <c r="J11" s="24" t="inlineStr"/>
+      <c r="K11" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/mc20-mini</t>
         </is>
       </c>
-      <c r="L11" s="4" t="inlineStr"/>
-      <c r="M11" s="4" t="inlineStr">
+      <c r="L11" s="24" t="inlineStr"/>
+      <c r="M11" s="24" t="inlineStr"/>
+      <c r="N11" s="24" t="inlineStr">
+        <is>
+          <t>Sem CNH</t>
+        </is>
+      </c>
+      <c r="O11" s="26" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N11" s="4" t="inlineStr">
+      <c r="P11" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="7" t="n">
+    <row r="12" ht="52" customHeight="1">
+      <c r="A12" s="28" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="28" t="inlineStr">
         <is>
           <t>MC21 Mini</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="28" t="inlineStr">
         <is>
           <t>Autopropelidos</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="28" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="28" t="inlineStr">
         <is>
           <t>1000 W</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F12" s="28" t="inlineStr">
         <is>
           <t>40 km</t>
         </is>
       </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>Equilíbrio perfeito entre design minimalista e desempenho elétrico. Bateria de lítio removível.</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
+      <c r="G12" s="29" t="inlineStr">
+        <is>
+          <t>Equilíbrio perfeito entre design minimalista e desempenho elétrico. Bateria de lítio removível e carregamento em casa.</t>
+        </is>
+      </c>
+      <c r="H12" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/mc21_mini_tin.webp</t>
         </is>
       </c>
-      <c r="I12" s="8" t="inlineStr"/>
-      <c r="J12" s="8" t="inlineStr"/>
-      <c r="K12" s="8" t="inlineStr">
+      <c r="I12" s="28" t="inlineStr"/>
+      <c r="J12" s="28" t="inlineStr"/>
+      <c r="K12" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/mc21-mini</t>
         </is>
       </c>
-      <c r="L12" s="7" t="inlineStr"/>
-      <c r="M12" s="7" t="inlineStr">
+      <c r="L12" s="28" t="inlineStr"/>
+      <c r="M12" s="28" t="inlineStr"/>
+      <c r="N12" s="28" t="inlineStr">
+        <is>
+          <t>Sem CNH</t>
+        </is>
+      </c>
+      <c r="O12" s="30" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N12" s="7" t="inlineStr">
+      <c r="P12" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="4" t="n">
+    <row r="13" ht="52" customHeight="1">
+      <c r="A13" s="24" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Mia</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="24" t="inlineStr">
         <is>
           <t>Autopropelidos</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="24" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="24" t="inlineStr">
         <is>
           <t>1000 W</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" s="24" t="inlineStr">
         <is>
           <t>40 km</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>Não é necessária CNH para conduzir um equipamento autopropelido (Resolução nº 996/2023 do Contran).</t>
-        </is>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="G13" s="25" t="inlineStr">
+        <is>
+          <t>Sem CNH, sem emplacamento. Resolução nº 996/2023 do Contran garante circulação legal. Motor 1000W e bateria removível.</t>
+        </is>
+      </c>
+      <c r="H13" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/10/MIA-1-1.webp</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr"/>
-      <c r="J13" s="5" t="inlineStr"/>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="I13" s="24" t="inlineStr"/>
+      <c r="J13" s="24" t="inlineStr"/>
+      <c r="K13" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/mia</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr"/>
-      <c r="M13" s="4" t="inlineStr">
+      <c r="L13" s="24" t="inlineStr"/>
+      <c r="M13" s="24" t="inlineStr"/>
+      <c r="N13" s="24" t="inlineStr">
+        <is>
+          <t>Sem CNH</t>
+        </is>
+      </c>
+      <c r="O13" s="26" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N13" s="4" t="inlineStr">
+      <c r="P13" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="7" t="n">
+    <row r="14" ht="52" customHeight="1">
+      <c r="A14" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="28" t="inlineStr">
         <is>
           <t>Sofia</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="28" t="inlineStr">
         <is>
           <t>Autopropelidos</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="28" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="28" t="inlineStr">
         <is>
           <t>1000 W</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F14" s="28" t="inlineStr">
         <is>
           <t>40 km</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
-        <is>
-          <t>Combina estilo clássico e tecnologia moderna. Motor 1000W, 32 km/h e autonomia de até 40 km.</t>
-        </is>
-      </c>
-      <c r="H14" s="8" t="inlineStr">
+      <c r="G14" s="29" t="inlineStr">
+        <is>
+          <t>Estilo clássico com tecnologia moderna. Motor 1000W, bateria removível e visual que agrada a todos os públicos.</t>
+        </is>
+      </c>
+      <c r="H14" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/sofia_web3_tiny.webp</t>
         </is>
       </c>
-      <c r="I14" s="8" t="inlineStr"/>
-      <c r="J14" s="8" t="inlineStr"/>
-      <c r="K14" s="8" t="inlineStr">
+      <c r="I14" s="28" t="inlineStr"/>
+      <c r="J14" s="28" t="inlineStr"/>
+      <c r="K14" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/sofia</t>
         </is>
       </c>
-      <c r="L14" s="7" t="inlineStr"/>
-      <c r="M14" s="7" t="inlineStr">
+      <c r="L14" s="28" t="inlineStr"/>
+      <c r="M14" s="28" t="inlineStr"/>
+      <c r="N14" s="28" t="inlineStr">
+        <is>
+          <t>Sem CNH</t>
+        </is>
+      </c>
+      <c r="O14" s="30" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N14" s="7" t="inlineStr">
+      <c r="P14" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="4" t="n">
+    <row r="15" ht="52" customHeight="1">
+      <c r="A15" s="24" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="24" t="inlineStr">
         <is>
           <t>Ret</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="24" t="inlineStr">
         <is>
           <t>Autopropelidos</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="24" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="24" t="inlineStr">
         <is>
           <t>1000 W</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F15" s="24" t="inlineStr">
         <is>
           <t>40 km</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>Visual agressivo, zero burocracia: ligou, acelerou, chegou.</t>
-        </is>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="G15" s="25" t="inlineStr">
+        <is>
+          <t>Estética retrô com motor 1000W e bateria de lítio. Presença de moto grande, praticidade de elétrica, sem burocracia.</t>
+        </is>
+      </c>
+      <c r="H15" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/10/RET-1-1.webp</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="5" t="inlineStr"/>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="I15" s="24" t="inlineStr"/>
+      <c r="J15" s="24" t="inlineStr"/>
+      <c r="K15" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/ret</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr"/>
-      <c r="M15" s="4" t="inlineStr">
+      <c r="L15" s="24" t="inlineStr"/>
+      <c r="M15" s="24" t="inlineStr"/>
+      <c r="N15" s="24" t="inlineStr">
+        <is>
+          <t>Sem CNH</t>
+        </is>
+      </c>
+      <c r="O15" s="26" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N15" s="4" t="inlineStr">
+      <c r="P15" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="7" t="n">
+    <row r="16" ht="52" customHeight="1">
+      <c r="A16" s="28" t="n">
         <v>14</v>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="28" t="inlineStr">
         <is>
           <t>Soma</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C16" s="28" t="inlineStr">
         <is>
           <t>Autopropelidos</t>
         </is>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="28" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="28" t="inlineStr">
         <is>
           <t>1000 W</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F16" s="28" t="inlineStr">
         <is>
           <t>40 km</t>
         </is>
       </c>
-      <c r="G16" s="9" t="inlineStr">
-        <is>
-          <t>Sem CNH, sem emplacamento. Motor 1000W, bateria 60V 20Ah removível e 40 km de autonomia.</t>
-        </is>
-      </c>
-      <c r="H16" s="8" t="inlineStr">
+      <c r="G16" s="29" t="inlineStr">
+        <is>
+          <t>Sem CNH, sem emplacamento. Motor 1000W, bateria 60V 20Ah removível e 40 km de autonomia por carga.</t>
+        </is>
+      </c>
+      <c r="H16" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/10/Soma-1-1-1.webp</t>
         </is>
       </c>
-      <c r="I16" s="8" t="inlineStr"/>
-      <c r="J16" s="8" t="inlineStr"/>
-      <c r="K16" s="8" t="inlineStr">
+      <c r="I16" s="28" t="inlineStr"/>
+      <c r="J16" s="28" t="inlineStr"/>
+      <c r="K16" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/soma</t>
         </is>
       </c>
-      <c r="L16" s="7" t="inlineStr"/>
-      <c r="M16" s="7" t="inlineStr">
+      <c r="L16" s="28" t="inlineStr"/>
+      <c r="M16" s="28" t="inlineStr"/>
+      <c r="N16" s="28" t="inlineStr">
+        <is>
+          <t>Sem CNH</t>
+        </is>
+      </c>
+      <c r="O16" s="30" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N16" s="7" t="inlineStr">
+      <c r="P16" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="4" t="n">
+    <row r="17" ht="52" customHeight="1">
+      <c r="A17" s="24" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="24" t="inlineStr">
         <is>
           <t>Mia Tri</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Autopropelidos</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="C17" s="24" t="inlineStr">
+        <is>
+          <t>Autopropelidos, Triciclos</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="24" t="inlineStr">
         <is>
           <t>800 W</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F17" s="24" t="inlineStr">
         <is>
           <t>40 km</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>Triciclo elétrico 800W para quem quer segurança, praticidade e estilo.</t>
-        </is>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="G17" s="25" t="inlineStr">
+        <is>
+          <t>Triciclo elétrico 800W para quem quer segurança extra, praticidade urbana e estilo moderno. Sem CNH.</t>
+        </is>
+      </c>
+      <c r="H17" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/10/MIA-TRI-01-1.webp</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr"/>
-      <c r="J17" s="5" t="inlineStr"/>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="I17" s="24" t="inlineStr"/>
+      <c r="J17" s="24" t="inlineStr"/>
+      <c r="K17" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/mia-tri</t>
         </is>
       </c>
-      <c r="L17" s="4" t="inlineStr"/>
-      <c r="M17" s="4" t="inlineStr">
+      <c r="L17" s="24" t="inlineStr"/>
+      <c r="M17" s="24" t="inlineStr"/>
+      <c r="N17" s="24" t="inlineStr">
+        <is>
+          <t>Sem CNH | Triciclo</t>
+        </is>
+      </c>
+      <c r="O17" s="26" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N17" s="4" t="inlineStr">
+      <c r="P17" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="7" t="n">
+    <row r="18" ht="52" customHeight="1">
+      <c r="A18" s="28" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="28" t="inlineStr">
         <is>
           <t>Joy Tri</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
-        <is>
-          <t>Autopropelidos</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="C18" s="28" t="inlineStr">
+        <is>
+          <t>Autopropelidos, Triciclos</t>
+        </is>
+      </c>
+      <c r="D18" s="28" t="inlineStr">
         <is>
           <t>30 km/h</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E18" s="28" t="inlineStr">
         <is>
           <t>600 W</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="F18" s="28" t="inlineStr">
         <is>
           <t>40 km</t>
         </is>
       </c>
-      <c r="G18" s="9" t="inlineStr">
-        <is>
-          <t>Chassi robusto de três rodas com estabilidade e confiança para o dia a dia.</t>
-        </is>
-      </c>
-      <c r="H18" s="8" t="inlineStr">
+      <c r="G18" s="29" t="inlineStr">
+        <is>
+          <t>Chassi de três rodas com estabilidade total. Ideal para quem quer segurança sem abrir mão da liberdade elétrica.</t>
+        </is>
+      </c>
+      <c r="H18" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/10/JOY-TRI-1-1.webp</t>
         </is>
       </c>
-      <c r="I18" s="8" t="inlineStr"/>
-      <c r="J18" s="8" t="inlineStr"/>
-      <c r="K18" s="8" t="inlineStr">
+      <c r="I18" s="28" t="inlineStr"/>
+      <c r="J18" s="28" t="inlineStr"/>
+      <c r="K18" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/joy-tri</t>
         </is>
       </c>
-      <c r="L18" s="7" t="inlineStr"/>
-      <c r="M18" s="7" t="inlineStr">
+      <c r="L18" s="28" t="inlineStr"/>
+      <c r="M18" s="28" t="inlineStr"/>
+      <c r="N18" s="28" t="inlineStr">
+        <is>
+          <t>Sem CNH | Triciclo</t>
+        </is>
+      </c>
+      <c r="O18" s="30" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N18" s="7" t="inlineStr">
+      <c r="P18" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="4" t="n">
+    <row r="19" ht="52" customHeight="1">
+      <c r="A19" s="24" t="n">
         <v>17</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>BIG TRI</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Autopropelidos</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="C19" s="24" t="inlineStr">
+        <is>
+          <t>Autopropelidos, Triciclos</t>
+        </is>
+      </c>
+      <c r="D19" s="24" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="24" t="inlineStr">
         <is>
           <t>1000 W</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F19" s="24" t="inlineStr">
         <is>
           <t>40 km</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>Liberdade com segurança. Design retrô, conforto e tecnologia moderna em triciclo elétrico 1000W.</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="G19" s="25" t="inlineStr">
+        <is>
+          <t>Liberdade com segurança. Design retrô, conforto ampliado e tecnologia elétrica moderna. Motor 1000W, sem CNH.</t>
+        </is>
+      </c>
+      <c r="H19" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/big_tri.webp</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr"/>
-      <c r="J19" s="5" t="inlineStr"/>
-      <c r="K19" s="5" t="inlineStr">
+      <c r="I19" s="24" t="inlineStr"/>
+      <c r="J19" s="24" t="inlineStr"/>
+      <c r="K19" s="24" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/big-tri/</t>
         </is>
       </c>
-      <c r="L19" s="4" t="inlineStr"/>
-      <c r="M19" s="4" t="inlineStr">
+      <c r="L19" s="24" t="inlineStr"/>
+      <c r="M19" s="24" t="inlineStr"/>
+      <c r="N19" s="24" t="inlineStr">
+        <is>
+          <t>Sem CNH | Triciclo</t>
+        </is>
+      </c>
+      <c r="O19" s="26" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N19" s="4" t="inlineStr">
+      <c r="P19" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="7" t="n">
+    <row r="20" ht="52" customHeight="1">
+      <c r="A20" s="28" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="28" t="inlineStr">
         <is>
           <t>VED</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>Autopropelidos</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="C20" s="28" t="inlineStr">
+        <is>
+          <t>Autopropelidos, Triciclos</t>
+        </is>
+      </c>
+      <c r="D20" s="28" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E20" s="28" t="inlineStr">
         <is>
           <t>1000 W</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F20" s="28" t="inlineStr">
         <is>
           <t>40 km</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
-        <is>
-          <t>Mobilidade elétrica acessível, segura e confortável. Motor 1000W e autonomia de até 40 km.</t>
-        </is>
-      </c>
-      <c r="H20" s="8" t="inlineStr">
+      <c r="G20" s="29" t="inlineStr">
+        <is>
+          <t>Mobilidade elétrica acessível e confortável. Motor 1000W, chassi de três rodas e autonomia de até 40 km. Sem CNH.</t>
+        </is>
+      </c>
+      <c r="H20" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/ved_1-1.webp</t>
         </is>
       </c>
-      <c r="I20" s="8" t="inlineStr"/>
-      <c r="J20" s="8" t="inlineStr"/>
-      <c r="K20" s="8" t="inlineStr">
+      <c r="I20" s="28" t="inlineStr"/>
+      <c r="J20" s="28" t="inlineStr"/>
+      <c r="K20" s="28" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/ved</t>
         </is>
       </c>
-      <c r="L20" s="7" t="inlineStr"/>
-      <c r="M20" s="7" t="inlineStr">
+      <c r="L20" s="28" t="inlineStr"/>
+      <c r="M20" s="28" t="inlineStr"/>
+      <c r="N20" s="28" t="inlineStr">
+        <is>
+          <t>Sem CNH | Triciclo</t>
+        </is>
+      </c>
+      <c r="O20" s="30" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N20" s="7" t="inlineStr">
+      <c r="P20" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="4" t="n">
+    <row r="21" ht="52" customHeight="1">
+      <c r="A21" s="31" t="n">
         <v>19</v>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="31" t="inlineStr">
         <is>
           <t>X11</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="31" t="inlineStr">
         <is>
           <t>Ciclomotor</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="31" t="inlineStr">
         <is>
           <t>50 km/h</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="31" t="inlineStr">
         <is>
           <t>2000 W</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F21" s="31" t="inlineStr">
         <is>
           <t>80 km</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>Design robusto e presença marcante com soluções modernas de mobilidade elétrica.</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="G21" s="32" t="inlineStr">
+        <is>
+          <t>Design robusto e presença marcante. Motor 2000W, até 80 km de autonomia — o mais completo da categoria ciclomotor.</t>
+        </is>
+      </c>
+      <c r="H21" s="31" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/x11__-1.webp</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr"/>
-      <c r="J21" s="5" t="inlineStr"/>
-      <c r="K21" s="5" t="inlineStr">
+      <c r="I21" s="31" t="inlineStr"/>
+      <c r="J21" s="31" t="inlineStr"/>
+      <c r="K21" s="31" t="inlineStr">
         <is>
           <t>https://motochefebrasil.com.br/modelos/x11</t>
         </is>
       </c>
-      <c r="L21" s="4" t="inlineStr"/>
-      <c r="M21" s="4" t="inlineStr">
+      <c r="L21" s="31" t="inlineStr"/>
+      <c r="M21" s="31" t="inlineStr"/>
+      <c r="N21" s="31" t="inlineStr">
+        <is>
+          <t>Maior Autonomia</t>
+        </is>
+      </c>
+      <c r="O21" s="33" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="P21" s="27" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="52" customHeight="1">
+      <c r="A22" s="31" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="31" t="inlineStr">
+        <is>
+          <t>MC20</t>
+        </is>
+      </c>
+      <c r="C22" s="31" t="inlineStr">
+        <is>
+          <t>Ciclomotor</t>
+        </is>
+      </c>
+      <c r="D22" s="31" t="inlineStr">
+        <is>
+          <t>50 km/h</t>
+        </is>
+      </c>
+      <c r="E22" s="31" t="inlineStr">
+        <is>
+          <t>2000 W</t>
+        </is>
+      </c>
+      <c r="F22" s="31" t="inlineStr">
+        <is>
+          <t>40 km</t>
+        </is>
+      </c>
+      <c r="G22" s="32" t="inlineStr">
+        <is>
+          <t>2000W ou 3000W, NFC, alarme com bloqueio, painel digital e até 80 km com bateria extra. Visual chopper, IP65.</t>
+        </is>
+      </c>
+      <c r="H22" s="31" t="inlineStr">
+        <is>
+          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/mc20_pop-1.webp</t>
+        </is>
+      </c>
+      <c r="I22" s="31" t="inlineStr"/>
+      <c r="J22" s="31" t="inlineStr"/>
+      <c r="K22" s="31" t="inlineStr">
+        <is>
+          <t>https://motochefebrasil.com.br/modelos/mc20/</t>
+        </is>
+      </c>
+      <c r="L22" s="31" t="inlineStr"/>
+      <c r="M22" s="31" t="inlineStr"/>
+      <c r="N22" s="31" t="inlineStr">
+        <is>
+          <t>NFC + Alarme</t>
+        </is>
+      </c>
+      <c r="O22" s="33" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="P22" s="27" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="52" customHeight="1">
+      <c r="A23" s="24" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>X15</t>
+        </is>
+      </c>
+      <c r="C23" s="24" t="inlineStr">
+        <is>
+          <t>Ciclomotor, Triciclos</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="inlineStr">
+        <is>
+          <t>50 km/h</t>
+        </is>
+      </c>
+      <c r="E23" s="24" t="inlineStr">
+        <is>
+          <t>3000 W</t>
+        </is>
+      </c>
+      <c r="F23" s="24" t="inlineStr">
+        <is>
+          <t>40 km</t>
+        </is>
+      </c>
+      <c r="G23" s="25" t="inlineStr">
+        <is>
+          <t>Triciclo elétrico potente. Motor 3000W para aceleração firme e desempenho consistente em qualquer pista.</t>
+        </is>
+      </c>
+      <c r="H23" s="24" t="inlineStr">
+        <is>
+          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/x15.webp</t>
+        </is>
+      </c>
+      <c r="I23" s="24" t="inlineStr"/>
+      <c r="J23" s="24" t="inlineStr"/>
+      <c r="K23" s="24" t="inlineStr">
+        <is>
+          <t>https://motochefebrasil.com.br/modelos/x15</t>
+        </is>
+      </c>
+      <c r="L23" s="24" t="inlineStr"/>
+      <c r="M23" s="24" t="inlineStr"/>
+      <c r="N23" s="24" t="inlineStr">
+        <is>
+          <t>Mais Potente</t>
+        </is>
+      </c>
+      <c r="O23" s="26" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N21" s="4" t="inlineStr">
+      <c r="P23" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="22" customHeight="1">
-      <c r="A22" s="7" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>MC20</t>
-        </is>
-      </c>
-      <c r="C22" s="7" t="inlineStr">
+    <row r="24" ht="52" customHeight="1">
+      <c r="A24" s="31" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="31" t="inlineStr">
+        <is>
+          <t>Roma</t>
+        </is>
+      </c>
+      <c r="C24" s="31" t="inlineStr">
         <is>
           <t>Ciclomotor</t>
         </is>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D24" s="31" t="inlineStr">
         <is>
           <t>50 km/h</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>2000 W</t>
-        </is>
-      </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>40 km</t>
-        </is>
-      </c>
-      <c r="G22" s="9" t="inlineStr">
-        <is>
-          <t>2000W ou 3000W, NFC, alarme com bloqueio, painel digital e até 80 km com bateria extra. Visual chopper, IP65.</t>
-        </is>
-      </c>
-      <c r="H22" s="8" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/mc20_pop-1.webp</t>
-        </is>
-      </c>
-      <c r="I22" s="8" t="inlineStr"/>
-      <c r="J22" s="8" t="inlineStr"/>
-      <c r="K22" s="8" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/modelos/mc20/</t>
-        </is>
-      </c>
-      <c r="L22" s="7" t="inlineStr"/>
-      <c r="M22" s="7" t="inlineStr">
+      <c r="E24" s="31" t="inlineStr">
+        <is>
+          <t>3000 W</t>
+        </is>
+      </c>
+      <c r="F24" s="31" t="inlineStr">
+        <is>
+          <t>50 km</t>
+        </is>
+      </c>
+      <c r="G24" s="32" t="inlineStr">
+        <is>
+          <t>Charme retrô europeu com tecnologia elétrica moderna. Motor 3000W, 50 km de autonomia e visual inconfundível.</t>
+        </is>
+      </c>
+      <c r="H24" s="31" t="inlineStr">
+        <is>
+          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/roma_ai_sombra-1.webp</t>
+        </is>
+      </c>
+      <c r="I24" s="31" t="inlineStr"/>
+      <c r="J24" s="31" t="inlineStr"/>
+      <c r="K24" s="31" t="inlineStr">
+        <is>
+          <t>https://motochefebrasil.com.br/modelos/roma</t>
+        </is>
+      </c>
+      <c r="L24" s="31" t="inlineStr"/>
+      <c r="M24" s="31" t="inlineStr"/>
+      <c r="N24" s="31" t="inlineStr">
+        <is>
+          <t>Design Premium</t>
+        </is>
+      </c>
+      <c r="O24" s="33" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="P24" s="27" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="52" customHeight="1">
+      <c r="A25" s="24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>GRID</t>
+        </is>
+      </c>
+      <c r="C25" s="24" t="inlineStr">
+        <is>
+          <t>E-Bikes</t>
+        </is>
+      </c>
+      <c r="D25" s="24" t="inlineStr">
+        <is>
+          <t>32 km/h</t>
+        </is>
+      </c>
+      <c r="E25" s="24" t="inlineStr">
+        <is>
+          <t>750 W</t>
+        </is>
+      </c>
+      <c r="F25" s="24" t="inlineStr">
+        <is>
+          <t>35 km</t>
+        </is>
+      </c>
+      <c r="G25" s="25" t="inlineStr">
+        <is>
+          <t>E-bike urbana ágil, robusta e divertida de pilotar. Motor 750W, freio a disco e bateria removível.</t>
+        </is>
+      </c>
+      <c r="H25" s="24" t="inlineStr">
+        <is>
+          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/10/GRID-LATERAL1-1.webp</t>
+        </is>
+      </c>
+      <c r="I25" s="24" t="inlineStr"/>
+      <c r="J25" s="24" t="inlineStr"/>
+      <c r="K25" s="24" t="inlineStr">
+        <is>
+          <t>https://motochefebrasil.com.br/modelos/grid/</t>
+        </is>
+      </c>
+      <c r="L25" s="24" t="inlineStr"/>
+      <c r="M25" s="24" t="inlineStr"/>
+      <c r="N25" s="24" t="inlineStr">
+        <is>
+          <t>Pedal Assistido</t>
+        </is>
+      </c>
+      <c r="O25" s="26" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N22" s="7" t="inlineStr">
+      <c r="P25" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>X15</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Ciclomotor</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>50 km/h</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>3000 W</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>40 km</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>Triciclo elétrico potente e seguro com motor 3000W para aceleração firme e desempenho consistente.</t>
-        </is>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/x15.webp</t>
-        </is>
-      </c>
-      <c r="I23" s="5" t="inlineStr"/>
-      <c r="J23" s="5" t="inlineStr"/>
-      <c r="K23" s="5" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/modelos/x15</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr"/>
-      <c r="M23" s="4" t="inlineStr">
+    <row r="26" ht="52" customHeight="1">
+      <c r="A26" s="31" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="31" t="inlineStr">
+        <is>
+          <t>Style</t>
+        </is>
+      </c>
+      <c r="C26" s="31" t="inlineStr">
+        <is>
+          <t>E-Bikes</t>
+        </is>
+      </c>
+      <c r="D26" s="31" t="inlineStr">
+        <is>
+          <t>32 km/h</t>
+        </is>
+      </c>
+      <c r="E26" s="31" t="inlineStr">
+        <is>
+          <t>750 W</t>
+        </is>
+      </c>
+      <c r="F26" s="31" t="inlineStr">
+        <is>
+          <t>35 km</t>
+        </is>
+      </c>
+      <c r="G26" s="32" t="inlineStr">
+        <is>
+          <t>E-bike urbana 750W (pico 1000W), bateria 48V 15,6Ah removível, freio a disco hidráulico — assinada por Diego Ribas.</t>
+        </is>
+      </c>
+      <c r="H26" s="31" t="inlineStr">
+        <is>
+          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/style-1-1.webp</t>
+        </is>
+      </c>
+      <c r="I26" s="31" t="inlineStr"/>
+      <c r="J26" s="31" t="inlineStr"/>
+      <c r="K26" s="31" t="inlineStr">
+        <is>
+          <t>https://motochefebrasil.com.br/modelos/style</t>
+        </is>
+      </c>
+      <c r="L26" s="31" t="inlineStr"/>
+      <c r="M26" s="31" t="inlineStr"/>
+      <c r="N26" s="31" t="inlineStr">
+        <is>
+          <t>Edição Diego Ribas</t>
+        </is>
+      </c>
+      <c r="O26" s="33" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="P26" s="27" t="inlineStr">
+        <is>
+          <t>Ativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="52" customHeight="1">
+      <c r="A27" s="24" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>Liberty</t>
+        </is>
+      </c>
+      <c r="C27" s="24" t="inlineStr">
+        <is>
+          <t>E-Bikes</t>
+        </is>
+      </c>
+      <c r="D27" s="24" t="inlineStr">
+        <is>
+          <t>32 km/h</t>
+        </is>
+      </c>
+      <c r="E27" s="24" t="inlineStr">
+        <is>
+          <t>500 W</t>
+        </is>
+      </c>
+      <c r="F27" s="24" t="inlineStr">
+        <is>
+          <t>35 km</t>
+        </is>
+      </c>
+      <c r="G27" s="25" t="inlineStr">
+        <is>
+          <t>Motor 500W (pico 800W), bateria 48V 13Ah removível e modos por aceleração ou pedal assistido PAS 5 níveis.</t>
+        </is>
+      </c>
+      <c r="H27" s="24" t="inlineStr">
+        <is>
+          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/liberty_product_web.webp</t>
+        </is>
+      </c>
+      <c r="I27" s="24" t="inlineStr"/>
+      <c r="J27" s="24" t="inlineStr"/>
+      <c r="K27" s="24" t="inlineStr">
+        <is>
+          <t>https://motochefebrasil.com.br/modelos/liberty</t>
+        </is>
+      </c>
+      <c r="L27" s="24" t="inlineStr"/>
+      <c r="M27" s="24" t="inlineStr"/>
+      <c r="N27" s="24" t="inlineStr">
+        <is>
+          <t>Pedal Assistido</t>
+        </is>
+      </c>
+      <c r="O27" s="26" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N23" s="4" t="inlineStr">
+      <c r="P27" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>Roma</t>
-        </is>
-      </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>Ciclomotor</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>50 km/h</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>3000 W</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>50 km</t>
-        </is>
-      </c>
-      <c r="G24" s="9" t="inlineStr">
-        <is>
-          <t>Charme retrô europeu com tecnologia elétrica moderna. 3000W, 50 km de autonomia.</t>
-        </is>
-      </c>
-      <c r="H24" s="8" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/roma_ai_sombra-1.webp</t>
-        </is>
-      </c>
-      <c r="I24" s="8" t="inlineStr"/>
-      <c r="J24" s="8" t="inlineStr"/>
-      <c r="K24" s="8" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/modelos/roma</t>
-        </is>
-      </c>
-      <c r="L24" s="7" t="inlineStr"/>
-      <c r="M24" s="7" t="inlineStr">
+    <row r="28" ht="52" customHeight="1">
+      <c r="A28" s="28" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="28" t="inlineStr">
+        <is>
+          <t>SPACE</t>
+        </is>
+      </c>
+      <c r="C28" s="28" t="inlineStr">
+        <is>
+          <t>E-Bikes</t>
+        </is>
+      </c>
+      <c r="D28" s="28" t="inlineStr">
+        <is>
+          <t>32 km/h</t>
+        </is>
+      </c>
+      <c r="E28" s="28" t="inlineStr">
+        <is>
+          <t>750 W</t>
+        </is>
+      </c>
+      <c r="F28" s="28" t="inlineStr">
+        <is>
+          <t>35 km</t>
+        </is>
+      </c>
+      <c r="G28" s="29" t="inlineStr">
+        <is>
+          <t>Motor 750W, bateria 48V 12Ah removível, 7 marchas. Aceleração no punho ou pedal assistido PAS 5 níveis.</t>
+        </is>
+      </c>
+      <c r="H28" s="28" t="inlineStr">
+        <is>
+          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/space_ia-1.webp</t>
+        </is>
+      </c>
+      <c r="I28" s="28" t="inlineStr"/>
+      <c r="J28" s="28" t="inlineStr"/>
+      <c r="K28" s="28" t="inlineStr">
+        <is>
+          <t>https://motochefebrasil.com.br/modelos/space</t>
+        </is>
+      </c>
+      <c r="L28" s="28" t="inlineStr"/>
+      <c r="M28" s="28" t="inlineStr"/>
+      <c r="N28" s="28" t="inlineStr">
+        <is>
+          <t>Pedal Assistido</t>
+        </is>
+      </c>
+      <c r="O28" s="30" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N24" s="7" t="inlineStr">
+      <c r="P28" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>GRID</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
+    <row r="29" ht="52" customHeight="1">
+      <c r="A29" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="24" t="inlineStr">
+        <is>
+          <t>Retrô</t>
+        </is>
+      </c>
+      <c r="C29" s="24" t="inlineStr">
         <is>
           <t>E-Bikes</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D29" s="24" t="inlineStr">
         <is>
           <t>32 km/h</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>750 W</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="E29" s="24" t="inlineStr">
+        <is>
+          <t>500 W</t>
+        </is>
+      </c>
+      <c r="F29" s="24" t="inlineStr">
         <is>
           <t>35 km</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>Ágil, robusta e divertida de pilotar.</t>
-        </is>
-      </c>
-      <c r="H25" s="5" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/10/GRID-LATERAL1-1.webp</t>
-        </is>
-      </c>
-      <c r="I25" s="5" t="inlineStr"/>
-      <c r="J25" s="5" t="inlineStr"/>
-      <c r="K25" s="5" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/modelos/grid/</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr"/>
-      <c r="M25" s="4" t="inlineStr">
+      <c r="G29" s="25" t="inlineStr">
+        <is>
+          <t>Visual de bike urbana clássica com praticidade de e-bike moderna. Motor 500W, pedal assistido e bateria removível.</t>
+        </is>
+      </c>
+      <c r="H29" s="24" t="inlineStr">
+        <is>
+          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/retro_hero-1.webp</t>
+        </is>
+      </c>
+      <c r="I29" s="24" t="inlineStr"/>
+      <c r="J29" s="24" t="inlineStr"/>
+      <c r="K29" s="24" t="inlineStr">
+        <is>
+          <t>https://motochefebrasil.com.br/modelos/retro</t>
+        </is>
+      </c>
+      <c r="L29" s="24" t="inlineStr"/>
+      <c r="M29" s="24" t="inlineStr"/>
+      <c r="N29" s="24" t="inlineStr">
+        <is>
+          <t>Pedal Assistido</t>
+        </is>
+      </c>
+      <c r="O29" s="26" t="inlineStr">
         <is>
           <t>Não</t>
         </is>
       </c>
-      <c r="N25" s="4" t="inlineStr">
+      <c r="P29" s="27" t="inlineStr">
         <is>
           <t>Ativo</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="7" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>Style</t>
-        </is>
-      </c>
-      <c r="C26" s="7" t="inlineStr">
-        <is>
-          <t>E-Bikes</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="inlineStr">
-        <is>
-          <t>32 km/h</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>750 W</t>
-        </is>
-      </c>
-      <c r="F26" s="7" t="inlineStr">
-        <is>
-          <t>35 km</t>
-        </is>
-      </c>
-      <c r="G26" s="9" t="inlineStr">
-        <is>
-          <t>E-bike urbana 750W (pico 1000W), bateria 48V 15,6Ah removível, freio a disco hidráulico — assinada por Diego Ribas.</t>
-        </is>
-      </c>
-      <c r="H26" s="8" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/style-1-1.webp</t>
-        </is>
-      </c>
-      <c r="I26" s="8" t="inlineStr"/>
-      <c r="J26" s="8" t="inlineStr"/>
-      <c r="K26" s="8" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/modelos/style</t>
-        </is>
-      </c>
-      <c r="L26" s="7" t="inlineStr"/>
-      <c r="M26" s="7" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="N26" s="7" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="22" customHeight="1">
-      <c r="A27" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>Liberty</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>E-Bikes</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>32 km/h</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>500 W</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>35 km</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>Motor 500W (pico 800W), bateria 48V 13Ah removível e modos por aceleração ou pedal assistido PAS 5 níveis.</t>
-        </is>
-      </c>
-      <c r="H27" s="5" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/liberty_product_web.webp</t>
-        </is>
-      </c>
-      <c r="I27" s="5" t="inlineStr"/>
-      <c r="J27" s="5" t="inlineStr"/>
-      <c r="K27" s="5" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/modelos/liberty</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr"/>
-      <c r="M27" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="N27" s="4" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="7" t="n">
-        <v>26</v>
-      </c>
-      <c r="B28" s="8" t="inlineStr">
-        <is>
-          <t>SPACE</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>E-Bikes</t>
-        </is>
-      </c>
-      <c r="D28" s="7" t="inlineStr">
-        <is>
-          <t>32 km/h</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>750 W</t>
-        </is>
-      </c>
-      <c r="F28" s="7" t="inlineStr">
-        <is>
-          <t>35 km</t>
-        </is>
-      </c>
-      <c r="G28" s="9" t="inlineStr">
-        <is>
-          <t>Motor 750W, bateria 48V 12Ah removível, 7 marchas. Aceleração no punho ou pedal assistido PAS 5 níveis.</t>
-        </is>
-      </c>
-      <c r="H28" s="8" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/space_ia-1.webp</t>
-        </is>
-      </c>
-      <c r="I28" s="8" t="inlineStr"/>
-      <c r="J28" s="8" t="inlineStr"/>
-      <c r="K28" s="8" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/modelos/space</t>
-        </is>
-      </c>
-      <c r="L28" s="7" t="inlineStr"/>
-      <c r="M28" s="7" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="N28" s="7" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="22" customHeight="1">
-      <c r="A29" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Retrô</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>E-Bikes</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>32 km/h</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>500 W</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>35 km</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>Visual de bike urbana com praticidade de e-bike moderna. Motor 500W, 32 km/h e 35 km de autonomia.</t>
-        </is>
-      </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/retro_hero-1.webp</t>
-        </is>
-      </c>
-      <c r="I29" s="5" t="inlineStr"/>
-      <c r="J29" s="5" t="inlineStr"/>
-      <c r="K29" s="5" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/modelos/retro</t>
-        </is>
-      </c>
-      <c r="L29" s="4" t="inlineStr"/>
-      <c r="M29" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="N29" s="4" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
-    </row>
     <row r="30" ht="22" customHeight="1">
-      <c r="A30" s="7" t="n">
-        <v>28</v>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>Joy Tri</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>Triciclos</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="inlineStr">
-        <is>
-          <t>30 km/h</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>600 W</t>
-        </is>
-      </c>
-      <c r="F30" s="7" t="inlineStr">
-        <is>
-          <t>40 km</t>
-        </is>
-      </c>
-      <c r="G30" s="9" t="inlineStr">
-        <is>
-          <t>Chassi de três rodas com estabilidade e confiança. Ideal para quem quer segurança sem abrir mão da liberdade.</t>
-        </is>
-      </c>
-      <c r="H30" s="8" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/10/JOY-TRI-1-1.webp</t>
-        </is>
-      </c>
-      <c r="I30" s="8" t="inlineStr"/>
-      <c r="J30" s="8" t="inlineStr"/>
-      <c r="K30" s="8" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/modelos/joy-tri</t>
-        </is>
-      </c>
-      <c r="L30" s="7" t="inlineStr"/>
-      <c r="M30" s="7" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="N30" s="7" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
+      <c r="A30" s="7" t="n"/>
+      <c r="B30" s="8" t="n"/>
+      <c r="C30" s="7" t="n"/>
+      <c r="D30" s="7" t="n"/>
+      <c r="E30" s="7" t="n"/>
+      <c r="F30" s="7" t="n"/>
+      <c r="G30" s="9" t="n"/>
+      <c r="H30" s="8" t="n"/>
+      <c r="I30" s="8" t="n"/>
+      <c r="J30" s="8" t="n"/>
+      <c r="K30" s="8" t="n"/>
+      <c r="L30" s="7" t="n"/>
+      <c r="M30" s="7" t="n"/>
+      <c r="N30" s="7" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="4" t="n">
-        <v>29</v>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>BIG TRI</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Triciclos</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>32 km/h</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>1000 W</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>40 km</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>Liberdade com segurança. Triciclo 1000W com design retrô, conforto e tecnologia moderna.</t>
-        </is>
-      </c>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/big_tri.webp</t>
-        </is>
-      </c>
-      <c r="I31" s="5" t="inlineStr"/>
-      <c r="J31" s="5" t="inlineStr"/>
-      <c r="K31" s="5" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/modelos/big-tri/</t>
-        </is>
-      </c>
-      <c r="L31" s="4" t="inlineStr"/>
-      <c r="M31" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="N31" s="4" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
+      <c r="A31" s="4" t="n"/>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="4" t="n"/>
+      <c r="D31" s="4" t="n"/>
+      <c r="E31" s="4" t="n"/>
+      <c r="F31" s="4" t="n"/>
+      <c r="G31" s="6" t="n"/>
+      <c r="H31" s="5" t="n"/>
+      <c r="I31" s="5" t="n"/>
+      <c r="J31" s="5" t="n"/>
+      <c r="K31" s="5" t="n"/>
+      <c r="L31" s="4" t="n"/>
+      <c r="M31" s="4" t="n"/>
+      <c r="N31" s="4" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="B32" s="8" t="inlineStr">
-        <is>
-          <t>Mia Tri</t>
-        </is>
-      </c>
-      <c r="C32" s="7" t="inlineStr">
-        <is>
-          <t>Triciclos</t>
-        </is>
-      </c>
-      <c r="D32" s="7" t="inlineStr">
-        <is>
-          <t>32 km/h</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="inlineStr">
-        <is>
-          <t>800 W</t>
-        </is>
-      </c>
-      <c r="F32" s="7" t="inlineStr">
-        <is>
-          <t>40 km</t>
-        </is>
-      </c>
-      <c r="G32" s="9" t="inlineStr">
-        <is>
-          <t>Triciclo elétrico 800W para quem quer segurança, praticidade e estilo.</t>
-        </is>
-      </c>
-      <c r="H32" s="8" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/10/MIA-TRI-01-1.webp</t>
-        </is>
-      </c>
-      <c r="I32" s="8" t="inlineStr"/>
-      <c r="J32" s="8" t="inlineStr"/>
-      <c r="K32" s="8" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/modelos/mia-tri</t>
-        </is>
-      </c>
-      <c r="L32" s="7" t="inlineStr"/>
-      <c r="M32" s="7" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="N32" s="7" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
+      <c r="A32" s="7" t="n"/>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="7" t="n"/>
+      <c r="D32" s="7" t="n"/>
+      <c r="E32" s="7" t="n"/>
+      <c r="F32" s="7" t="n"/>
+      <c r="G32" s="9" t="n"/>
+      <c r="H32" s="8" t="n"/>
+      <c r="I32" s="8" t="n"/>
+      <c r="J32" s="8" t="n"/>
+      <c r="K32" s="8" t="n"/>
+      <c r="L32" s="7" t="n"/>
+      <c r="M32" s="7" t="n"/>
+      <c r="N32" s="7" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="4" t="n">
-        <v>31</v>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>X15</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>Triciclos</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>50 km/h</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>3000 W</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>40 km</t>
-        </is>
-      </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>Triciclo elétrico potente com motor 3000W para aceleração firme e desempenho consistente.</t>
-        </is>
-      </c>
-      <c r="H33" s="5" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/x15.webp</t>
-        </is>
-      </c>
-      <c r="I33" s="5" t="inlineStr"/>
-      <c r="J33" s="5" t="inlineStr"/>
-      <c r="K33" s="5" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/modelos/x15</t>
-        </is>
-      </c>
-      <c r="L33" s="4" t="inlineStr"/>
-      <c r="M33" s="4" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="N33" s="4" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
+      <c r="A33" s="4" t="n"/>
+      <c r="B33" s="5" t="n"/>
+      <c r="C33" s="4" t="n"/>
+      <c r="D33" s="4" t="n"/>
+      <c r="E33" s="4" t="n"/>
+      <c r="F33" s="4" t="n"/>
+      <c r="G33" s="6" t="n"/>
+      <c r="H33" s="5" t="n"/>
+      <c r="I33" s="5" t="n"/>
+      <c r="J33" s="5" t="n"/>
+      <c r="K33" s="5" t="n"/>
+      <c r="L33" s="4" t="n"/>
+      <c r="M33" s="4" t="n"/>
+      <c r="N33" s="4" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
-      <c r="A34" s="7" t="n">
-        <v>32</v>
-      </c>
-      <c r="B34" s="8" t="inlineStr">
-        <is>
-          <t>VED</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>Triciclos</t>
-        </is>
-      </c>
-      <c r="D34" s="7" t="inlineStr">
-        <is>
-          <t>32 km/h</t>
-        </is>
-      </c>
-      <c r="E34" s="7" t="inlineStr">
-        <is>
-          <t>1000 W</t>
-        </is>
-      </c>
-      <c r="F34" s="7" t="inlineStr">
-        <is>
-          <t>40 km</t>
-        </is>
-      </c>
-      <c r="G34" s="9" t="inlineStr">
-        <is>
-          <t>Mobilidade elétrica acessível, segura e confortável. Motor 1000W e autonomia de até 40 km.</t>
-        </is>
-      </c>
-      <c r="H34" s="8" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/wp-content/uploads/2025/11/ved_1-1.webp</t>
-        </is>
-      </c>
-      <c r="I34" s="8" t="inlineStr"/>
-      <c r="J34" s="8" t="inlineStr"/>
-      <c r="K34" s="8" t="inlineStr">
-        <is>
-          <t>https://motochefebrasil.com.br/modelos/ved</t>
-        </is>
-      </c>
-      <c r="L34" s="7" t="inlineStr"/>
-      <c r="M34" s="7" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="N34" s="7" t="inlineStr">
-        <is>
-          <t>Ativo</t>
-        </is>
-      </c>
+      <c r="A34" s="7" t="n"/>
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="7" t="n"/>
+      <c r="E34" s="7" t="n"/>
+      <c r="F34" s="7" t="n"/>
+      <c r="G34" s="9" t="n"/>
+      <c r="H34" s="8" t="n"/>
+      <c r="I34" s="8" t="n"/>
+      <c r="J34" s="8" t="n"/>
+      <c r="K34" s="8" t="n"/>
+      <c r="L34" s="7" t="n"/>
+      <c r="M34" s="7" t="n"/>
+      <c r="N34" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2563,7 +2661,7 @@
       <formula>$M3="Sim"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
+  <dataValidations count="6">
     <dataValidation sqref="C3:C84" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Categoria inválida" error="Escolha da lista." type="list">
       <formula1>"Autopropelidos,Ciclomotor,E-Bikes,Triciclos"</formula1>
     </dataValidation>
@@ -2572,6 +2670,15 @@
     </dataValidation>
     <dataValidation sqref="N3:N84" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Status inválido" error="Escolha da lista." type="list">
       <formula1>"Ativo,Inativo,Rascunho"</formula1>
+    </dataValidation>
+    <dataValidation sqref="O3:O100" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Valor invalido" error="Escolha Sim ou Nao" type="list">
+      <formula1>"Sim,Nao"</formula1>
+    </dataValidation>
+    <dataValidation sqref="P3:P100" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Valor invalido" error="Escolha Ativo ou Inativo" type="list">
+      <formula1>"Ativo,Inativo"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C3:C100" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Categoria invalida" error="Escolha uma categoria da lista" type="list">
+      <formula1>"Autopropelidos,Ciclomotor,E-Bikes,Triciclos,Autopropelidos; Triciclos,Ciclomotor; Triciclos"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2606,6 +2713,8 @@
           <t>🔑  IDENTIFICAÇÃO</t>
         </is>
       </c>
+      <c r="C3" s="34" t="n"/>
+      <c r="D3" s="35" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="B4" s="11" t="inlineStr">
@@ -2664,6 +2773,8 @@
           <t>⚙️  ESPECIFICAÇÕES (exibidas no pop-up)</t>
         </is>
       </c>
+      <c r="C8" s="34" t="n"/>
+      <c r="D8" s="35" t="n"/>
     </row>
     <row r="9" ht="24" customHeight="1">
       <c r="B9" s="11" t="inlineStr">
@@ -2722,6 +2833,8 @@
           <t>📝  CONTEÚDO</t>
         </is>
       </c>
+      <c r="C13" s="34" t="n"/>
+      <c r="D13" s="35" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1">
       <c r="B14" s="11" t="inlineStr">
@@ -2746,6 +2859,8 @@
           <t>🖼️  IMAGENS</t>
         </is>
       </c>
+      <c r="C16" s="34" t="n"/>
+      <c r="D16" s="35" t="n"/>
     </row>
     <row r="17" ht="24" customHeight="1">
       <c r="B17" s="11" t="inlineStr">
@@ -2804,6 +2919,8 @@
           <t>🌐  LINK</t>
         </is>
       </c>
+      <c r="C21" s="34" t="n"/>
+      <c r="D21" s="35" t="n"/>
     </row>
     <row r="22" ht="24" customHeight="1">
       <c r="B22" s="11" t="inlineStr">
@@ -2828,6 +2945,8 @@
           <t>💰  PREÇO</t>
         </is>
       </c>
+      <c r="C24" s="34" t="n"/>
+      <c r="D24" s="35" t="n"/>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="B25" s="11" t="inlineStr">
@@ -2852,6 +2971,8 @@
           <t>🎯  SELETOR DE OFERTA — IMPORTANTE</t>
         </is>
       </c>
+      <c r="C27" s="34" t="n"/>
+      <c r="D27" s="35" t="n"/>
     </row>
     <row r="28" ht="24" customHeight="1">
       <c r="B28" s="11" t="inlineStr">
@@ -2877,6 +2998,8 @@
           <t>📦  CONTROLE</t>
         </is>
       </c>
+      <c r="C30" s="34" t="n"/>
+      <c r="D30" s="35" t="n"/>
     </row>
     <row r="31" ht="24" customHeight="1">
       <c r="B31" s="11" t="inlineStr">
@@ -2901,6 +3024,8 @@
           <t>⚠️  DICAS RÁPIDAS</t>
         </is>
       </c>
+      <c r="C34" s="34" t="n"/>
+      <c r="D34" s="35" t="n"/>
     </row>
     <row r="35" ht="22" customHeight="1">
       <c r="B35" s="15" t="inlineStr">
@@ -2908,6 +3033,8 @@
           <t xml:space="preserve">  •  Cada linha = 1 produto no catálogo do site</t>
         </is>
       </c>
+      <c r="C35" s="34" t="n"/>
+      <c r="D35" s="35" t="n"/>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="B36" s="15" t="inlineStr">
@@ -2915,6 +3042,8 @@
           <t xml:space="preserve">  •  Cada coluna = 1 campo do pop-up do produto</t>
         </is>
       </c>
+      <c r="C36" s="34" t="n"/>
+      <c r="D36" s="35" t="n"/>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="B37" s="15" t="inlineStr">
@@ -2922,6 +3051,8 @@
           <t xml:space="preserve">  •  Para adicionar novo produto: copie a última linha e edite</t>
         </is>
       </c>
+      <c r="C37" s="34" t="n"/>
+      <c r="D37" s="35" t="n"/>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="B38" s="15" t="inlineStr">
@@ -2929,6 +3060,8 @@
           <t xml:space="preserve">  •  ID deve ser único — nunca repita o mesmo número</t>
         </is>
       </c>
+      <c r="C38" s="34" t="n"/>
+      <c r="D38" s="35" t="n"/>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="B39" s="15" t="inlineStr">
@@ -2936,6 +3069,8 @@
           <t xml:space="preserve">  •  Use Status = Inativo para ocultar sem excluir</t>
         </is>
       </c>
+      <c r="C39" s="34" t="n"/>
+      <c r="D39" s="35" t="n"/>
     </row>
     <row r="40" ht="22" customHeight="1">
       <c r="B40" s="15" t="inlineStr">
@@ -2943,6 +3078,8 @@
           <t xml:space="preserve">  •  A Imagem Destaque é a foto principal visível no card — use sempre a melhor foto</t>
         </is>
       </c>
+      <c r="C40" s="34" t="n"/>
+      <c r="D40" s="35" t="n"/>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="B41" s="15" t="inlineStr">
@@ -2950,6 +3087,8 @@
           <t xml:space="preserve">  •  Ao marcar Oferta = Sim, a linha fica destacada automaticamente em amarelo nesta planilha</t>
         </is>
       </c>
+      <c r="C41" s="34" t="n"/>
+      <c r="D41" s="35" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="17">
@@ -2963,10 +3102,10 @@
     <mergeCell ref="B40:D40"/>
     <mergeCell ref="B27:D27"/>
     <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B38:D38"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="B30:D30"/>
     <mergeCell ref="B39:D39"/>
-    <mergeCell ref="B38:D38"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B34:D34"/>

</xml_diff>